<commit_message>
Daily routine trscker 2
</commit_message>
<xml_diff>
--- a/12618140.xlsx
+++ b/12618140.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -202,6 +202,18 @@
   </si>
   <si>
     <t>I felt tired after last two class.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Satisfied </t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>I felt good after all class.</t>
   </si>
 </sst>
 </file>
@@ -1024,26 +1036,49 @@
       </c>
     </row>
     <row r="7" spans="1:14">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="15" t="str">
-        <f t="shared" ref="I7:I69" si="0">IF(SUM(B7:F7,H7)=0,"",SUM(B7:F7,H7))</f>
-        <v/>
-      </c>
-      <c r="J7" s="15" t="str">
-        <f t="shared" ref="J6:J69" si="1">IF(I7="","",1440-I7)</f>
-        <v/>
-      </c>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="17"/>
+      <c r="A7" s="13">
+        <v>46247</v>
+      </c>
+      <c r="B7" s="14">
+        <v>450</v>
+      </c>
+      <c r="C7" s="14">
+        <v>50</v>
+      </c>
+      <c r="D7" s="14">
+        <v>120</v>
+      </c>
+      <c r="E7" s="14">
+        <v>60</v>
+      </c>
+      <c r="F7" s="14">
+        <v>150</v>
+      </c>
+      <c r="G7" s="14">
+        <v>3</v>
+      </c>
+      <c r="H7" s="14">
+        <v>120</v>
+      </c>
+      <c r="I7" s="15">
+        <v>950</v>
+      </c>
+      <c r="J7" s="15">
+        <f t="shared" ref="J7:J69" si="0">IF(I7="","",1440-I7)</f>
+        <v>490</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="13"/>
@@ -1055,11 +1090,11 @@
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
       <c r="I8" s="15" t="str">
+        <f t="shared" ref="I7:I69" si="1">IF(SUM(B8:F8,H8)=0,"",SUM(B8:F8,H8))</f>
+        <v/>
+      </c>
+      <c r="J8" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K8" s="16"/>
@@ -1077,11 +1112,11 @@
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
       <c r="I9" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J9" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K9" s="16"/>
@@ -1099,11 +1134,11 @@
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
       <c r="I10" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J10" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K10" s="16"/>
@@ -1121,11 +1156,11 @@
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
       <c r="I11" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J11" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K11" s="16"/>
@@ -1143,11 +1178,11 @@
       <c r="G12" s="14"/>
       <c r="H12" s="14"/>
       <c r="I12" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J12" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K12" s="16"/>
@@ -1165,11 +1200,11 @@
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
       <c r="I13" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J13" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K13" s="16"/>
@@ -1187,11 +1222,11 @@
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
       <c r="I14" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J14" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K14" s="16"/>
@@ -1209,11 +1244,11 @@
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
       <c r="I15" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J15" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K15" s="16"/>
@@ -1231,11 +1266,11 @@
       <c r="G16" s="14"/>
       <c r="H16" s="14"/>
       <c r="I16" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J16" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K16" s="16"/>
@@ -1253,11 +1288,11 @@
       <c r="G17" s="14"/>
       <c r="H17" s="14"/>
       <c r="I17" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J17" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K17" s="16"/>
@@ -1275,11 +1310,11 @@
       <c r="G18" s="14"/>
       <c r="H18" s="14"/>
       <c r="I18" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J18" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K18" s="16"/>
@@ -1297,11 +1332,11 @@
       <c r="G19" s="14"/>
       <c r="H19" s="14"/>
       <c r="I19" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J19" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K19" s="16"/>
@@ -1319,11 +1354,11 @@
       <c r="G20" s="14"/>
       <c r="H20" s="14"/>
       <c r="I20" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J20" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K20" s="16"/>
@@ -1341,11 +1376,11 @@
       <c r="G21" s="14"/>
       <c r="H21" s="14"/>
       <c r="I21" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J21" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K21" s="16"/>
@@ -1363,11 +1398,11 @@
       <c r="G22" s="14"/>
       <c r="H22" s="14"/>
       <c r="I22" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J22" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K22" s="16"/>
@@ -1385,11 +1420,11 @@
       <c r="G23" s="14"/>
       <c r="H23" s="14"/>
       <c r="I23" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J23" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K23" s="16"/>
@@ -1407,11 +1442,11 @@
       <c r="G24" s="14"/>
       <c r="H24" s="14"/>
       <c r="I24" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J24" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K24" s="16"/>
@@ -1429,11 +1464,11 @@
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
       <c r="I25" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J25" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K25" s="16"/>
@@ -1451,11 +1486,11 @@
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J26" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K26" s="16"/>
@@ -1473,11 +1508,11 @@
       <c r="G27" s="14"/>
       <c r="H27" s="14"/>
       <c r="I27" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J27" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K27" s="16"/>
@@ -1495,11 +1530,11 @@
       <c r="G28" s="14"/>
       <c r="H28" s="14"/>
       <c r="I28" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J28" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K28" s="16"/>
@@ -1517,11 +1552,11 @@
       <c r="G29" s="14"/>
       <c r="H29" s="14"/>
       <c r="I29" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J29" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K29" s="16"/>
@@ -1539,11 +1574,11 @@
       <c r="G30" s="14"/>
       <c r="H30" s="14"/>
       <c r="I30" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J30" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K30" s="16"/>
@@ -1561,11 +1596,11 @@
       <c r="G31" s="14"/>
       <c r="H31" s="14"/>
       <c r="I31" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J31" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K31" s="16"/>
@@ -1583,11 +1618,11 @@
       <c r="G32" s="14"/>
       <c r="H32" s="14"/>
       <c r="I32" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J32" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K32" s="16"/>
@@ -1605,11 +1640,11 @@
       <c r="G33" s="14"/>
       <c r="H33" s="14"/>
       <c r="I33" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J33" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K33" s="16"/>
@@ -1627,11 +1662,11 @@
       <c r="G34" s="14"/>
       <c r="H34" s="14"/>
       <c r="I34" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J34" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K34" s="16"/>
@@ -1649,11 +1684,11 @@
       <c r="G35" s="14"/>
       <c r="H35" s="14"/>
       <c r="I35" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J35" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K35" s="16"/>
@@ -1671,11 +1706,11 @@
       <c r="G36" s="14"/>
       <c r="H36" s="14"/>
       <c r="I36" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J36" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K36" s="16"/>
@@ -1693,11 +1728,11 @@
       <c r="G37" s="14"/>
       <c r="H37" s="14"/>
       <c r="I37" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J37" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K37" s="16"/>
@@ -1715,11 +1750,11 @@
       <c r="G38" s="14"/>
       <c r="H38" s="14"/>
       <c r="I38" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J38" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K38" s="16"/>
@@ -1737,11 +1772,11 @@
       <c r="G39" s="14"/>
       <c r="H39" s="14"/>
       <c r="I39" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J39" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K39" s="16"/>
@@ -1759,11 +1794,11 @@
       <c r="G40" s="14"/>
       <c r="H40" s="14"/>
       <c r="I40" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J40" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K40" s="16"/>
@@ -1781,11 +1816,11 @@
       <c r="G41" s="14"/>
       <c r="H41" s="14"/>
       <c r="I41" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J41" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K41" s="16"/>
@@ -1803,11 +1838,11 @@
       <c r="G42" s="14"/>
       <c r="H42" s="14"/>
       <c r="I42" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J42" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K42" s="16"/>
@@ -1825,11 +1860,11 @@
       <c r="G43" s="14"/>
       <c r="H43" s="14"/>
       <c r="I43" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J43" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K43" s="16"/>
@@ -1847,11 +1882,11 @@
       <c r="G44" s="14"/>
       <c r="H44" s="14"/>
       <c r="I44" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J44" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K44" s="16"/>
@@ -1869,11 +1904,11 @@
       <c r="G45" s="14"/>
       <c r="H45" s="14"/>
       <c r="I45" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J45" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K45" s="16"/>
@@ -1891,11 +1926,11 @@
       <c r="G46" s="14"/>
       <c r="H46" s="14"/>
       <c r="I46" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J46" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K46" s="16"/>
@@ -1913,11 +1948,11 @@
       <c r="G47" s="14"/>
       <c r="H47" s="14"/>
       <c r="I47" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J47" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K47" s="16"/>
@@ -1935,11 +1970,11 @@
       <c r="G48" s="14"/>
       <c r="H48" s="14"/>
       <c r="I48" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J48" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K48" s="16"/>
@@ -1957,11 +1992,11 @@
       <c r="G49" s="14"/>
       <c r="H49" s="14"/>
       <c r="I49" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J49" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K49" s="16"/>
@@ -1979,11 +2014,11 @@
       <c r="G50" s="14"/>
       <c r="H50" s="14"/>
       <c r="I50" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J50" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K50" s="16"/>
@@ -2001,11 +2036,11 @@
       <c r="G51" s="14"/>
       <c r="H51" s="14"/>
       <c r="I51" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J51" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K51" s="16"/>
@@ -2023,11 +2058,11 @@
       <c r="G52" s="14"/>
       <c r="H52" s="14"/>
       <c r="I52" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J52" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K52" s="16"/>
@@ -2045,11 +2080,11 @@
       <c r="G53" s="14"/>
       <c r="H53" s="14"/>
       <c r="I53" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J53" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K53" s="16"/>
@@ -2067,11 +2102,11 @@
       <c r="G54" s="14"/>
       <c r="H54" s="14"/>
       <c r="I54" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J54" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K54" s="16"/>
@@ -2089,11 +2124,11 @@
       <c r="G55" s="14"/>
       <c r="H55" s="14"/>
       <c r="I55" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J55" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K55" s="16"/>
@@ -2111,11 +2146,11 @@
       <c r="G56" s="14"/>
       <c r="H56" s="14"/>
       <c r="I56" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J56" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K56" s="16"/>
@@ -2133,11 +2168,11 @@
       <c r="G57" s="14"/>
       <c r="H57" s="14"/>
       <c r="I57" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J57" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K57" s="16"/>
@@ -2155,11 +2190,11 @@
       <c r="G58" s="14"/>
       <c r="H58" s="14"/>
       <c r="I58" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J58" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K58" s="16"/>
@@ -2177,11 +2212,11 @@
       <c r="G59" s="14"/>
       <c r="H59" s="14"/>
       <c r="I59" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J59" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K59" s="16"/>
@@ -2199,11 +2234,11 @@
       <c r="G60" s="14"/>
       <c r="H60" s="14"/>
       <c r="I60" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J60" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J60" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K60" s="16"/>
@@ -2221,11 +2256,11 @@
       <c r="G61" s="14"/>
       <c r="H61" s="14"/>
       <c r="I61" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J61" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J61" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K61" s="16"/>
@@ -2243,11 +2278,11 @@
       <c r="G62" s="14"/>
       <c r="H62" s="14"/>
       <c r="I62" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J62" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J62" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K62" s="16"/>
@@ -2265,11 +2300,11 @@
       <c r="G63" s="14"/>
       <c r="H63" s="14"/>
       <c r="I63" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J63" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J63" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K63" s="16"/>
@@ -2287,11 +2322,11 @@
       <c r="G64" s="14"/>
       <c r="H64" s="14"/>
       <c r="I64" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J64" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J64" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K64" s="16"/>
@@ -2309,11 +2344,11 @@
       <c r="G65" s="14"/>
       <c r="H65" s="14"/>
       <c r="I65" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J65" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J65" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K65" s="16"/>
@@ -2331,11 +2366,11 @@
       <c r="G66" s="14"/>
       <c r="H66" s="14"/>
       <c r="I66" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J66" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J66" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K66" s="16"/>
@@ -2353,11 +2388,11 @@
       <c r="G67" s="14"/>
       <c r="H67" s="14"/>
       <c r="I67" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J67" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J67" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K67" s="16"/>
@@ -2375,11 +2410,11 @@
       <c r="G68" s="14"/>
       <c r="H68" s="14"/>
       <c r="I68" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J68" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J68" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K68" s="16"/>
@@ -2397,11 +2432,11 @@
       <c r="G69" s="14"/>
       <c r="H69" s="14"/>
       <c r="I69" s="15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J69" s="15" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J69" s="15" t="str">
-        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="K69" s="16"/>

</xml_diff>